<commit_message>
fix: build the photo-gap workbook from the current run, not a stale coverage file
The "Photos Missing" sheet was reading photo_coverage_zip.csv left over from the
older PDF-based build, so articles the report writes with a leading zero never
matched and articles the PDF route had merged were missing entirely. The full
catalogue builder now writes that coverage itself, from the same pass that builds
the index, and the workbook matches the item code as written before falling back
to the normalised form.

Sort the sheet so the six articles that need a photo shoot come before the 45 that
only need a file renamed, and list the colours in stock so the shoot knows what to
cover.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Article-Photos-Missing.xlsx
+++ b/Article-Photos-Missing.xlsx
@@ -66,15 +66,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="5" max="5" width="34" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="7" max="7" width="26" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="52" customWidth="1"/>
+    <col min="9" max="9" width="58" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -100,7 +100,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Colours</t>
+          <t xml:space="preserve">Colours in stock</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -127,12 +127,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEAST-109</t>
+          <t xml:space="preserve">STAR GIRL DLX BUCKLE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEAST</t>
+          <t xml:space="preserve">STAR GIRL DLX BUCKLE</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -141,277 +141,291 @@
         </is>
       </c>
       <c r="D2">
-        <v>195</v>
-      </c>
-      <c r="E2">
-        <v>3</v>
+        <v>53</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BLK</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">11X1, 2X5</t>
+          <t xml:space="preserve">11X13, 1X3, 4X5, 6X8</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve">369.99, 399.99</t>
+          <t xml:space="preserve">259.99, 279.99, 319.99, 359.99</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SERIES ONLY</t>
+          <t xml:space="preserve">NO PHOTO</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAME A PHOTO - series folder has photos, none named for this article</t>
+          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SPEED-3</t>
+          <t xml:space="preserve">STAR GIRL-V DLX</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SPEED</t>
+          <t xml:space="preserve">STAR GIRL</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">STUCKON</t>
+          <t xml:space="preserve">VERTICAL</t>
         </is>
       </c>
       <c r="D3">
-        <v>130</v>
-      </c>
-      <c r="E3">
-        <v>3</v>
+        <v>49</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BLK</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">11X1, 2X5</t>
+          <t xml:space="preserve">1 NO, 11 NO, 11X13, 1X3, 2 NO, 4 NO, 4X5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve">729.99, 779.99, 829.99</t>
+          <t xml:space="preserve">259.99, 279.99, 319.99</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SERIES ONLY</t>
+          <t xml:space="preserve">NO PHOTO</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAME A PHOTO - series folder has photos, none named for this article</t>
+          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">EVA-GOLA-V-21</t>
+          <t xml:space="preserve">RABBIT</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">EVA</t>
+          <t xml:space="preserve">RABBIT</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">STUCKON</t>
+          <t xml:space="preserve">PU</t>
         </is>
       </c>
       <c r="D4">
-        <v>127</v>
-      </c>
-      <c r="E4">
-        <v>2</v>
+        <v>20</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B.PNK, DGR, T.BLU</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">11X1, 2X5, 4X5, 6X8, 8 NO, 8K, 8X10K, 9X10</t>
+          <t xml:space="preserve">5X10K</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">549.99, 579.99, 619.99, 659.99, 699.99</t>
+          <t xml:space="preserve">309.99</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve">SERIES ONLY</t>
+          <t xml:space="preserve">NO PHOTO</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAME A PHOTO - series folder has photos, none named for this article</t>
+          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">VENUS-01-PAD</t>
+          <t xml:space="preserve">SOLDIER</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">VENUS</t>
+          <t xml:space="preserve">SOLDIER</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">PU</t>
+          <t xml:space="preserve">EVA</t>
         </is>
       </c>
       <c r="D5">
-        <v>122</v>
-      </c>
-      <c r="E5">
-        <v>3</v>
+        <v>17</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MINT GRN, NBL, OFF WHT</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">11X1, 7X10K</t>
+          <t xml:space="preserve">11X13, 1X3, 4X7</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">499.99, 529.99</t>
+          <t xml:space="preserve">399, 449, 499</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">SERIES ONLY</t>
+          <t xml:space="preserve">NO PHOTO</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAME A PHOTO - series folder has photos, none named for this article</t>
+          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">EVA-GOLA-L-1</t>
+          <t xml:space="preserve">CUST SPORTS-42</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">EVA</t>
+          <t xml:space="preserve">CUST SPORTS</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">STUCKON</t>
+          <t xml:space="preserve">ROTARY</t>
         </is>
       </c>
       <c r="D6">
-        <v>122</v>
-      </c>
-      <c r="E6">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BLK</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">11X1, 2X5, 6X8, 9X10</t>
+          <t xml:space="preserve">11X1</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">589.99, 619.99, 629.99, 659.99, 699.99</t>
+          <t xml:space="preserve">389.99</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve">SERIES ONLY</t>
+          <t xml:space="preserve">NO PHOTO</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAME A PHOTO - series folder has photos, none named for this article</t>
+          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">STANLAY-3</t>
+          <t xml:space="preserve">GSJ-22-L</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">STANLAY</t>
+          <t xml:space="preserve">GSJ</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">EVA</t>
+          <t xml:space="preserve">STUCKON</t>
         </is>
       </c>
       <c r="D7">
-        <v>79</v>
-      </c>
-      <c r="E7">
         <v>1</v>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BLK/PNK</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">20X25K, 26X31, 32X35</t>
+          <t xml:space="preserve">5X8</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve">339.99, 379.99, 429.99</t>
+          <t xml:space="preserve">649</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t xml:space="preserve">SERIES ONLY</t>
+          <t xml:space="preserve">NO PHOTO</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAME A PHOTO - series folder has photos, none named for this article</t>
+          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ROME-1</t>
+          <t xml:space="preserve">BEAST-109</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ROME</t>
+          <t xml:space="preserve">BEAST</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">STUCKON</t>
+          <t xml:space="preserve">VERTICAL</t>
         </is>
       </c>
       <c r="D8">
-        <v>63</v>
-      </c>
-      <c r="E8">
-        <v>3</v>
+        <v>195</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BLK, DGR, OLV</t>
+        </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">11X1, 7X10K</t>
+          <t xml:space="preserve">11X1, 2X5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">599.99, 649.99</t>
+          <t xml:space="preserve">369.99, 399.99</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -428,33 +442,35 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">CRETA-11</t>
+          <t xml:space="preserve">KSJ-404</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">CRETA</t>
+          <t xml:space="preserve">KSJ</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">PU</t>
+          <t xml:space="preserve">STUCKON</t>
         </is>
       </c>
       <c r="D9">
-        <v>58</v>
-      </c>
-      <c r="E9">
-        <v>4</v>
+        <v>191</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BLK, LGR, T.BLU, TAN</t>
+        </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">5X8, 6X9</t>
+          <t xml:space="preserve">11X1, 2X5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t xml:space="preserve">519.99</t>
+          <t xml:space="preserve">619.99, 649.99, 659.99, 689.99</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -471,24 +487,26 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEAST-111</t>
+          <t xml:space="preserve">SPEED-3</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEAST</t>
+          <t xml:space="preserve">SPEED</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERTICAL</t>
+          <t xml:space="preserve">STUCKON</t>
         </is>
       </c>
       <c r="D10">
-        <v>56</v>
-      </c>
-      <c r="E10">
-        <v>3</v>
+        <v>130</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BEG, BNT, OLV</t>
+        </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -497,7 +515,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve">369.99, 399.99</t>
+          <t xml:space="preserve">729.99, 779.99, 829.99</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -514,33 +532,35 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSD-1601/CL</t>
+          <t xml:space="preserve">EVA-GOLA-V-21</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSD</t>
+          <t xml:space="preserve">EVA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">PU</t>
+          <t xml:space="preserve">STUCKON</t>
         </is>
       </c>
       <c r="D11">
-        <v>46</v>
-      </c>
-      <c r="E11">
-        <v>4</v>
+        <v>127</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BLK, WHT</t>
+        </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">11X1, 2X5, 5X10K</t>
+          <t xml:space="preserve">11X1, 2X5, 4X5, 6X8, 8 NO, 8K, 8X10K, 9X10</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve">239.99, 269.99, 299, 299.99</t>
+          <t xml:space="preserve">549.99, 579.99, 619.99, 659.99, 699.99</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -557,33 +577,35 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">VENUS-03-PAD</t>
+          <t xml:space="preserve">EVA-GOLA-L-1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">VENUS</t>
+          <t xml:space="preserve">EVA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">PU</t>
+          <t xml:space="preserve">STUCKON</t>
         </is>
       </c>
       <c r="D12">
-        <v>43</v>
-      </c>
-      <c r="E12">
-        <v>3</v>
+        <v>122</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BLK, WHT</t>
+        </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">11X1, 7X10K</t>
+          <t xml:space="preserve">11X1, 2X5, 6X8, 9X10</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve">499.99, 529.99</t>
+          <t xml:space="preserve">589.99, 619.99, 629.99, 659.99, 699.99</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -600,33 +622,35 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUKE-110</t>
+          <t xml:space="preserve">VENUS-01-PAD</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUKE</t>
+          <t xml:space="preserve">VENUS</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERTICAL</t>
+          <t xml:space="preserve">PU</t>
         </is>
       </c>
       <c r="D13">
-        <v>40</v>
-      </c>
-      <c r="E13">
-        <v>3</v>
+        <v>122</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BLK, NBL, T.BLU</t>
+        </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">5X10K</t>
+          <t xml:space="preserve">11X1, 7X10K</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve">299.99</t>
+          <t xml:space="preserve">499.99, 529.99</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -643,12 +667,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARS-9</t>
+          <t xml:space="preserve">SPEED-4</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARS</t>
+          <t xml:space="preserve">SPEED</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -657,10 +681,12 @@
         </is>
       </c>
       <c r="D14">
-        <v>34</v>
-      </c>
-      <c r="E14">
-        <v>1</v>
+        <v>117</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BEG, BNT, OLV</t>
+        </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -669,7 +695,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t xml:space="preserve">829.99, 879.99</t>
+          <t xml:space="preserve">729.99, 779.99, 829.99</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -686,24 +712,26 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">EAGLE-21-L</t>
+          <t xml:space="preserve">MARS-06</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">EAGLE</t>
+          <t xml:space="preserve">MARS</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">ROTARY</t>
+          <t xml:space="preserve">STUCKON</t>
         </is>
       </c>
       <c r="D15">
-        <v>32</v>
-      </c>
-      <c r="E15">
-        <v>1</v>
+        <v>86</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BEG, BNT, OLV</t>
+        </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -712,7 +740,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t xml:space="preserve">469.99, 499.99</t>
+          <t xml:space="preserve">799.99, 849.99, 899.99</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -729,33 +757,35 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">CANDY-121</t>
+          <t xml:space="preserve">STANLAY-3</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">CANDY</t>
+          <t xml:space="preserve">STANLAY</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERTICAL</t>
+          <t xml:space="preserve">EVA</t>
         </is>
       </c>
       <c r="D16">
-        <v>28</v>
-      </c>
-      <c r="E16">
-        <v>1</v>
+        <v>79</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LGR/NBL</t>
+        </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">4X7, 5X7, 5X8</t>
+          <t xml:space="preserve">20X25K, 26X31, 32X35</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t xml:space="preserve">409.99</t>
+          <t xml:space="preserve">339.99, 379.99, 429.99</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -772,33 +802,35 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">CRYSTA-03-L</t>
+          <t xml:space="preserve">ROME-1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">CRYSTA</t>
+          <t xml:space="preserve">ROME</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERTICAL</t>
+          <t xml:space="preserve">STUCKON</t>
         </is>
       </c>
       <c r="D17">
-        <v>26</v>
-      </c>
-      <c r="E17">
-        <v>1</v>
+        <v>63</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BLK, BNT, T.BLU</t>
+        </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve">4X7, 5X8</t>
+          <t xml:space="preserve">11X1, 7X10K</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t xml:space="preserve">429.99</t>
+          <t xml:space="preserve">599.99, 649.99</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -815,33 +847,35 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">KSJ-201(BLK-SOLE)</t>
+          <t xml:space="preserve">CRETA-11</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">KSJ</t>
+          <t xml:space="preserve">CRETA</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">STUCKON</t>
+          <t xml:space="preserve">PU</t>
         </is>
       </c>
       <c r="D18">
-        <v>26</v>
-      </c>
-      <c r="E18">
-        <v>1</v>
+        <v>58</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BLK, NBL, OLV, PPL</t>
+        </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">11X1, 2X5</t>
+          <t xml:space="preserve">5X8, 6X9</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t xml:space="preserve">579, 599</t>
+          <t xml:space="preserve">519.99</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -858,24 +892,26 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">KSJ-414</t>
+          <t xml:space="preserve">BEAST-111</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">KSJ</t>
+          <t xml:space="preserve">BEAST</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">STUCKON</t>
+          <t xml:space="preserve">VERTICAL</t>
         </is>
       </c>
       <c r="D19">
-        <v>17</v>
-      </c>
-      <c r="E19">
-        <v>2</v>
+        <v>56</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AFB, BEG, PST</t>
+        </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -884,7 +920,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t xml:space="preserve">659.99, 689.99</t>
+          <t xml:space="preserve">369.99, 399.99</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -901,33 +937,35 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">VENUS-02-PAD</t>
+          <t xml:space="preserve">KSJ-119</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">VENUS</t>
+          <t xml:space="preserve">KSJ</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">PU</t>
+          <t xml:space="preserve">STUCKON</t>
         </is>
       </c>
       <c r="D20">
-        <v>16</v>
-      </c>
-      <c r="E20">
-        <v>1</v>
+        <v>55</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LGR, NBL, WHT</t>
+        </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">11X1, 7X10K</t>
+          <t xml:space="preserve">11X1, 2X5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t xml:space="preserve">499.99, 529.99</t>
+          <t xml:space="preserve">549.99, 579.99, 589.99, 619.99</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -944,33 +982,35 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">STANLAY-205</t>
+          <t xml:space="preserve">GSD-1601/CL</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">STANLAY</t>
+          <t xml:space="preserve">GSD</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">EVA</t>
+          <t xml:space="preserve">PU</t>
         </is>
       </c>
       <c r="D21">
-        <v>14</v>
-      </c>
-      <c r="E21">
-        <v>1</v>
+        <v>46</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B.PNK, BLK, MRN, PST</t>
+        </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">20X25K, 26X31, 32X35</t>
+          <t xml:space="preserve">11X1, 2X5, 5X10K</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t xml:space="preserve">339.99, 379.99, 419.99</t>
+          <t xml:space="preserve">239.99, 269.99, 299, 299.99</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -987,12 +1027,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSD-1107/CL</t>
+          <t xml:space="preserve">VENUS-03-PAD</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSD</t>
+          <t xml:space="preserve">VENUS</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1001,19 +1041,21 @@
         </is>
       </c>
       <c r="D22">
-        <v>13</v>
-      </c>
-      <c r="E22">
-        <v>2</v>
+        <v>43</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DGR, NBL, T.BLU</t>
+        </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">2X5, 5X10K</t>
+          <t xml:space="preserve">11X1, 7X10K</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t xml:space="preserve">229, 229.99, 289, 289.99</t>
+          <t xml:space="preserve">499.99, 529.99</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1030,12 +1072,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">JSS-13</t>
+          <t xml:space="preserve">LUKE-110</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">JSS</t>
+          <t xml:space="preserve">LUKE</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1044,10 +1086,12 @@
         </is>
       </c>
       <c r="D23">
-        <v>11</v>
-      </c>
-      <c r="E23">
-        <v>1</v>
+        <v>40</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AFB, DGR, KHK</t>
+        </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1073,33 +1117,35 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">LITTLE-1(SHARK)</t>
+          <t xml:space="preserve">MARS-9</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">LITTLE</t>
+          <t xml:space="preserve">MARS</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">OUT SIDE</t>
+          <t xml:space="preserve">STUCKON</t>
         </is>
       </c>
       <c r="D24">
-        <v>9</v>
-      </c>
-      <c r="E24">
-        <v>3</v>
+        <v>34</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OLV</t>
+        </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">5X10K</t>
+          <t xml:space="preserve">11X1, 2X5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t xml:space="preserve">214.99</t>
+          <t xml:space="preserve">829.99, 879.99</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1116,33 +1162,35 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSD-250/CL</t>
+          <t xml:space="preserve">EAGLE-21-L</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSD</t>
+          <t xml:space="preserve">EAGLE</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">PU</t>
+          <t xml:space="preserve">ROTARY</t>
         </is>
       </c>
       <c r="D25">
-        <v>8</v>
-      </c>
-      <c r="E25">
-        <v>2</v>
+        <v>32</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OLV</t>
+        </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">2X5</t>
+          <t xml:space="preserve">11X1, 2X5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t xml:space="preserve">269, 269.99</t>
+          <t xml:space="preserve">469.99, 499.99</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1159,12 +1207,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">TODDLER-104</t>
+          <t xml:space="preserve">CANDY-11 L</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">TODDLER</t>
+          <t xml:space="preserve">CANDY</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1173,19 +1221,21 @@
         </is>
       </c>
       <c r="D26">
-        <v>7</v>
-      </c>
-      <c r="E26">
-        <v>2</v>
+        <v>31</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BLK</t>
+        </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">16X21</t>
+          <t xml:space="preserve">4X7, 5X8, 6X9</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t xml:space="preserve">219.99</t>
+          <t xml:space="preserve">409.99</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1202,12 +1252,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">SPORTS-56</t>
+          <t xml:space="preserve">CANDY-121</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">SPORTS</t>
+          <t xml:space="preserve">CANDY</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1216,19 +1266,21 @@
         </is>
       </c>
       <c r="D27">
-        <v>6</v>
-      </c>
-      <c r="E27">
-        <v>4</v>
+        <v>28</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MRN</t>
+        </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve">2X5</t>
+          <t xml:space="preserve">4X7, 5X7, 5X8</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t xml:space="preserve">389.99</t>
+          <t xml:space="preserve">409.99</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1245,33 +1297,35 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSD-263</t>
+          <t xml:space="preserve">CRYSTA-03-L</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSD</t>
+          <t xml:space="preserve">CRYSTA</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">PU</t>
+          <t xml:space="preserve">VERTICAL</t>
         </is>
       </c>
       <c r="D28">
-        <v>6</v>
-      </c>
-      <c r="E28">
-        <v>1</v>
+        <v>26</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BLK/BLK</t>
+        </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t xml:space="preserve">11X1, 2X5, 5X10K</t>
+          <t xml:space="preserve">4X7, 5X8</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t xml:space="preserve">219.99, 249.99, 279.99</t>
+          <t xml:space="preserve">429.99</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1288,24 +1342,26 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">ZOYA-05</t>
+          <t xml:space="preserve">KSJ-201(BLK-SOLE)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">ZOYA</t>
+          <t xml:space="preserve">KSJ</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">PU</t>
+          <t xml:space="preserve">STUCKON</t>
         </is>
       </c>
       <c r="D29">
-        <v>5</v>
-      </c>
-      <c r="E29">
-        <v>1</v>
+        <v>26</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BLK</t>
+        </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1314,7 +1370,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t xml:space="preserve">499.99, 529.99</t>
+          <t xml:space="preserve">579, 599</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1331,33 +1387,35 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUKE-7-L</t>
+          <t xml:space="preserve">ITALY-01 7X10</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUKE</t>
+          <t xml:space="preserve">ITALY</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERTICAL</t>
+          <t xml:space="preserve">STUCKON</t>
         </is>
       </c>
       <c r="D30">
-        <v>5</v>
-      </c>
-      <c r="E30">
-        <v>1</v>
+        <v>17</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RNI</t>
+        </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t xml:space="preserve">5X10K</t>
+          <t xml:space="preserve">7X10</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t xml:space="preserve">349.99</t>
+          <t xml:space="preserve">639.99</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1374,33 +1432,35 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">SONIC-51</t>
+          <t xml:space="preserve">KSJ-414</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">SONIC</t>
+          <t xml:space="preserve">KSJ</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERTICAL</t>
+          <t xml:space="preserve">STUCKON</t>
         </is>
       </c>
       <c r="D31">
-        <v>5</v>
-      </c>
-      <c r="E31">
-        <v>1</v>
+        <v>17</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BEG, NBL</t>
+        </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve">11X1</t>
+          <t xml:space="preserve">11X1, 2X5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t xml:space="preserve">469.99</t>
+          <t xml:space="preserve">659.99, 689.99</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1417,12 +1477,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">KSD-340-NEW</t>
+          <t xml:space="preserve">VENUS-02-PAD</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">KSD</t>
+          <t xml:space="preserve">VENUS</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1431,19 +1491,21 @@
         </is>
       </c>
       <c r="D32">
-        <v>4</v>
-      </c>
-      <c r="E32">
-        <v>2</v>
+        <v>16</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PPL</t>
+        </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2X5</t>
+          <t xml:space="preserve">11X1, 7X10K</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t xml:space="preserve">339.99</t>
+          <t xml:space="preserve">499.99, 529.99</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1460,33 +1522,35 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">KSJ-55-V</t>
+          <t xml:space="preserve">STANLAY-205</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">KSJ</t>
+          <t xml:space="preserve">STANLAY</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">STUCKON</t>
+          <t xml:space="preserve">EVA</t>
         </is>
       </c>
       <c r="D33">
-        <v>2</v>
-      </c>
-      <c r="E33">
-        <v>1</v>
+        <v>14</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LMN/MNT</t>
+        </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">11X1</t>
+          <t xml:space="preserve">20X25K, 26X31, 32X35</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t xml:space="preserve">569.99</t>
+          <t xml:space="preserve">339.99, 379.99, 419.99</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1503,33 +1567,35 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEAST-03</t>
+          <t xml:space="preserve">DIYA-02 PLUS</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEAST</t>
+          <t xml:space="preserve">DIYA</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERTICAL</t>
+          <t xml:space="preserve">STUCKON</t>
         </is>
       </c>
       <c r="D34">
-        <v>1</v>
-      </c>
-      <c r="E34">
-        <v>1</v>
+        <v>14</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KHK, OLV, PPL</t>
+        </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve">2X5</t>
+          <t xml:space="preserve">4X7</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t xml:space="preserve">409</t>
+          <t xml:space="preserve">649.99, 699.99</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1546,33 +1612,35 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">FIRE-2006</t>
+          <t xml:space="preserve">GSD-1107/CL</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">FIRE</t>
+          <t xml:space="preserve">GSD</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">AIR</t>
+          <t xml:space="preserve">PU</t>
         </is>
       </c>
       <c r="D35">
-        <v>1</v>
-      </c>
-      <c r="E35">
-        <v>1</v>
+        <v>13</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PCH, PISTA</t>
+        </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">36X41</t>
+          <t xml:space="preserve">2X5, 5X10K</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t xml:space="preserve">279</t>
+          <t xml:space="preserve">229, 229.99, 289, 289.99</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1589,33 +1657,35 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">CRETA-12</t>
+          <t xml:space="preserve">ITALY-102</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">CRETA</t>
+          <t xml:space="preserve">ITALY</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">PU</t>
+          <t xml:space="preserve">STUCKON</t>
         </is>
       </c>
       <c r="D36">
-        <v>1</v>
-      </c>
-      <c r="E36">
-        <v>1</v>
+        <v>12</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BNT, NBL, OLV</t>
+        </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t xml:space="preserve">5X8</t>
+          <t xml:space="preserve">2X5</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t xml:space="preserve">519.99</t>
+          <t xml:space="preserve">799.99</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1632,33 +1702,35 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">KSJ-413-V</t>
+          <t xml:space="preserve">JSS-13</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">KSJ</t>
+          <t xml:space="preserve">JSS</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">STUCKON</t>
+          <t xml:space="preserve">VERTICAL</t>
         </is>
       </c>
       <c r="D37">
-        <v>1</v>
-      </c>
-      <c r="E37">
-        <v>1</v>
+        <v>11</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OLV</t>
+        </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t xml:space="preserve">2X5</t>
+          <t xml:space="preserve">5X10K</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t xml:space="preserve">729.99</t>
+          <t xml:space="preserve">299.99</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1675,98 +1747,102 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAR BOY DLX-L</t>
+          <t xml:space="preserve">LITTLE-1(SHARK)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAR BOY DLX</t>
+          <t xml:space="preserve">LITTLE</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERTICAL</t>
+          <t xml:space="preserve">OUT SIDE</t>
         </is>
       </c>
       <c r="D38">
-        <v>368</v>
-      </c>
-      <c r="E38">
-        <v>2</v>
+        <v>9</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AQUA, NBL, OLV</t>
+        </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 K, 11K, 11X13, 1X3, 4 K, 4X5, 5, 6, 6X8, 8K, 8X10K, 9K, 9X10</t>
+          <t xml:space="preserve">5X10K</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t xml:space="preserve">249.99, 279.99, 289.99, 299.99, 329.99, 369.99, 379.99, 409.99, 469.99</t>
+          <t xml:space="preserve">214.99</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
+          <t xml:space="preserve">SERIES ONLY</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
+          <t xml:space="preserve">NAME A PHOTO - series folder has photos, none named for this article</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAR GOLA-L</t>
+          <t xml:space="preserve">GSD-250/CL</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAR GOLA</t>
+          <t xml:space="preserve">GSD</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERTICAL</t>
+          <t xml:space="preserve">PU</t>
         </is>
       </c>
       <c r="D39">
-        <v>249</v>
-      </c>
-      <c r="E39">
-        <v>1</v>
+        <v>8</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PCH, PST</t>
+        </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t xml:space="preserve">11X13, 1X3, 4 NO, 4X5, 5 NO, 6 NO, 7 NO, 8 NO, 8X10K</t>
+          <t xml:space="preserve">2X5</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t xml:space="preserve">379.99, 409.99, 449.99, 499.99, 549.99</t>
+          <t xml:space="preserve">269, 269.99</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
+          <t xml:space="preserve">SERIES ONLY</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
+          <t xml:space="preserve">NAME A PHOTO - series folder has photos, none named for this article</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAR GIRL BUCKLE PLAIN</t>
+          <t xml:space="preserve">TODDLER-104</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAR GIRL BUCKLE PLAIN</t>
+          <t xml:space="preserve">TODDLER</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1775,84 +1851,88 @@
         </is>
       </c>
       <c r="D40">
-        <v>239</v>
-      </c>
-      <c r="E40">
-        <v>1</v>
+        <v>7</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MHD, SBL</t>
+        </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 NO, 11X13, 12 NO, 1X3, 2 NO, 4X5, 6X8, 8X10K</t>
+          <t xml:space="preserve">16X21</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t xml:space="preserve">229.99, 249.99, 279.99, 309.99, 349.99</t>
+          <t xml:space="preserve">219.99</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
+          <t xml:space="preserve">SERIES ONLY</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
+          <t xml:space="preserve">NAME A PHOTO - series folder has photos, none named for this article</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAR OPEN BELLY PLAIN</t>
+          <t xml:space="preserve">GSD-263</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAR OPEN BELLY PLAIN</t>
+          <t xml:space="preserve">GSD</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERTICAL</t>
+          <t xml:space="preserve">PU</t>
         </is>
       </c>
       <c r="D41">
-        <v>230</v>
-      </c>
-      <c r="E41">
-        <v>1</v>
+        <v>6</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B.PNK</t>
+        </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">11X13, 1X3, 3 NO, 4X5, 6 NO, 6X8, 7 NO, 8 NO, 8X10K</t>
+          <t xml:space="preserve">11X1, 2X5, 5X10K</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t xml:space="preserve">199.99, 219.99, 239.99, 269.99, 299.99</t>
+          <t xml:space="preserve">219.99, 249.99, 279.99</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
+          <t xml:space="preserve">SERIES ONLY</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
+          <t xml:space="preserve">NAME A PHOTO - series folder has photos, none named for this article</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAR GOLA-V</t>
+          <t xml:space="preserve">SPORTS-56</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAR GOLA</t>
+          <t xml:space="preserve">SPORTS</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1861,84 +1941,88 @@
         </is>
       </c>
       <c r="D42">
-        <v>140</v>
-      </c>
-      <c r="E42">
-        <v>2</v>
+        <v>6</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AFB, DGR, KHK, OLV</t>
+        </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 NO, 11X13, 13 NO, 1X2, 1X3, 2 NO, 4 NO, 4X5, 6 NO, 6X8, 8X10K, 9K</t>
+          <t xml:space="preserve">2X5</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t xml:space="preserve">379.99, 409.99, 429.99, 449.99, 499.99, 529.99, 549.99, 579.99</t>
+          <t xml:space="preserve">389.99</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
+          <t xml:space="preserve">SERIES ONLY</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
+          <t xml:space="preserve">NAME A PHOTO - series folder has photos, none named for this article</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAR GIRL DLX FV</t>
+          <t xml:space="preserve">ZOYA-05</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAR GIRL DLX FV</t>
+          <t xml:space="preserve">ZOYA</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERTICAL</t>
+          <t xml:space="preserve">PU</t>
         </is>
       </c>
       <c r="D43">
-        <v>95</v>
-      </c>
-      <c r="E43">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PCH</t>
+        </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t xml:space="preserve">11X13, 1X3, 4X5, 6X7, 6X8, 8X10K</t>
+          <t xml:space="preserve">11X1, 2X5</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t xml:space="preserve">239.99, 259.99, 279.99, 289.99, 319.99, 359.99</t>
+          <t xml:space="preserve">499.99, 529.99</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
+          <t xml:space="preserve">SERIES ONLY</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
+          <t xml:space="preserve">NAME A PHOTO - series folder has photos, none named for this article</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAR BOY PLAIN-L</t>
+          <t xml:space="preserve">LUKE-7-L</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAR BOY PLAIN</t>
+          <t xml:space="preserve">LUKE</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1947,41 +2031,43 @@
         </is>
       </c>
       <c r="D44">
-        <v>77</v>
-      </c>
-      <c r="E44">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PNK</t>
+        </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t xml:space="preserve">11X13, 1X3, 4 NO, 4X5, 6X8, 8X10K, 9X10</t>
+          <t xml:space="preserve">5X10K</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t xml:space="preserve">229.99, 259.99, 289.99, 319.99, 359.99</t>
+          <t xml:space="preserve">349.99</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
+          <t xml:space="preserve">SERIES ONLY</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
+          <t xml:space="preserve">NAME A PHOTO - series folder has photos, none named for this article</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAR GIRL DLX BUCKLE</t>
+          <t xml:space="preserve">SONIC-51</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAR GIRL DLX BUCKLE</t>
+          <t xml:space="preserve">SONIC</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1990,170 +2076,178 @@
         </is>
       </c>
       <c r="D45">
-        <v>53</v>
-      </c>
-      <c r="E45">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOS</t>
+        </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t xml:space="preserve">11X13, 1X3, 4X5, 6X8</t>
+          <t xml:space="preserve">11X1</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t xml:space="preserve">259.99, 279.99, 319.99, 359.99</t>
+          <t xml:space="preserve">469.99</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
+          <t xml:space="preserve">SERIES ONLY</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
+          <t xml:space="preserve">NAME A PHOTO - series folder has photos, none named for this article</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAR GIRL-V DLX</t>
+          <t xml:space="preserve">KSD-340-NEW</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAR GIRL</t>
+          <t xml:space="preserve">KSD</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERTICAL</t>
+          <t xml:space="preserve">PU</t>
         </is>
       </c>
       <c r="D46">
-        <v>49</v>
-      </c>
-      <c r="E46">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BRN, N.PST</t>
+        </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 NO, 11 NO, 11X13, 1X3, 2 NO, 4 NO, 4X5</t>
+          <t xml:space="preserve">2X5</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t xml:space="preserve">259.99, 279.99, 319.99</t>
+          <t xml:space="preserve">339.99</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
+          <t xml:space="preserve">SERIES ONLY</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
+          <t xml:space="preserve">NAME A PHOTO - series folder has photos, none named for this article</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">CANDY-11 L</t>
+          <t xml:space="preserve">DIYA-08 6X9</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">CANDY</t>
+          <t xml:space="preserve">DIYA</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERTICAL</t>
+          <t xml:space="preserve">STUCKON</t>
         </is>
       </c>
       <c r="D47">
-        <v>31</v>
-      </c>
-      <c r="E47">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R.GOLD</t>
+        </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t xml:space="preserve">4X7, 5X8, 6X9</t>
+          <t xml:space="preserve">6X9</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t xml:space="preserve">409.99</t>
+          <t xml:space="preserve">639.99</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
+          <t xml:space="preserve">SERIES ONLY</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
+          <t xml:space="preserve">NAME A PHOTO - series folder has photos, none named for this article</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAR BOY DLX-V</t>
+          <t xml:space="preserve">KSJ-55-V</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAR BOY DLX</t>
+          <t xml:space="preserve">KSJ</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERTICAL</t>
+          <t xml:space="preserve">STUCKON</t>
         </is>
       </c>
       <c r="D48">
-        <v>23</v>
-      </c>
-      <c r="E48">
         <v>2</v>
       </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBL/SBL</t>
+        </is>
+      </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t xml:space="preserve">11X13, 1X3, 8X10K</t>
+          <t xml:space="preserve">11X1</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t xml:space="preserve">299.99, 329.99, 339.99, 359.99, 379.99</t>
+          <t xml:space="preserve">569.99</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
+          <t xml:space="preserve">SERIES ONLY</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
+          <t xml:space="preserve">NAME A PHOTO - series folder has photos, none named for this article</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">RABBIT</t>
+          <t xml:space="preserve">CRETA-12</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">RABBIT</t>
+          <t xml:space="preserve">CRETA</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2162,127 +2256,133 @@
         </is>
       </c>
       <c r="D49">
-        <v>20</v>
-      </c>
-      <c r="E49">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DGR</t>
+        </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t xml:space="preserve">5X10K</t>
+          <t xml:space="preserve">5X8</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t xml:space="preserve">309.99</t>
+          <t xml:space="preserve">519.99</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
+          <t xml:space="preserve">SERIES ONLY</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
+          <t xml:space="preserve">NAME A PHOTO - series folder has photos, none named for this article</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITALY-01 7X10</t>
+          <t xml:space="preserve">BEAST-03</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITALY</t>
+          <t xml:space="preserve">BEAST</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">STUCKON</t>
+          <t xml:space="preserve">VERTICAL</t>
         </is>
       </c>
       <c r="D50">
-        <v>17</v>
-      </c>
-      <c r="E50">
         <v>1</v>
       </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PISTA</t>
+        </is>
+      </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t xml:space="preserve">7X10</t>
+          <t xml:space="preserve">2X5</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t xml:space="preserve">639.99</t>
+          <t xml:space="preserve">409</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
+          <t xml:space="preserve">SERIES ONLY</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
+          <t xml:space="preserve">NAME A PHOTO - series folder has photos, none named for this article</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOLDIER</t>
+          <t xml:space="preserve">FIRE-2006</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOLDIER</t>
+          <t xml:space="preserve">FIRE</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">EVA</t>
+          <t xml:space="preserve">AIR</t>
         </is>
       </c>
       <c r="D51">
-        <v>17</v>
-      </c>
-      <c r="E51">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBL/NBL/WHT</t>
+        </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t xml:space="preserve">11X13, 1X3, 4X7</t>
+          <t xml:space="preserve">36X41</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t xml:space="preserve">399, 449, 499</t>
+          <t xml:space="preserve">279</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
+          <t xml:space="preserve">SERIES ONLY</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
+          <t xml:space="preserve">NAME A PHOTO - series folder has photos, none named for this article</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">DIYA-02 PLUS</t>
+          <t xml:space="preserve">KSJ-413-V</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">DIYA</t>
+          <t xml:space="preserve">KSJ</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2291,352 +2391,53 @@
         </is>
       </c>
       <c r="D52">
-        <v>14</v>
-      </c>
-      <c r="E52">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BEG</t>
+        </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t xml:space="preserve">4X7</t>
+          <t xml:space="preserve">2X5</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t xml:space="preserve">649.99, 699.99</t>
+          <t xml:space="preserve">729.99</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
+          <t xml:space="preserve">SERIES ONLY</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
+          <t xml:space="preserve">NAME A PHOTO - series folder has photos, none named for this article</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">FIRE BOLT-06</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FIRE BOLT</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VERTICAL</t>
-        </is>
-      </c>
+          <t xml:space="preserve">TOTAL</t>
+        </is>
+      </c>
+      <c r="B53"/>
+      <c r="C53"/>
       <c r="D53">
-        <v>9</v>
-      </c>
-      <c r="E53">
-        <v>2</v>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6X10K</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">449.99</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CUST SPORTS-42</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CUST SPORTS</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ROTARY</t>
-        </is>
-      </c>
-      <c r="D54">
-        <v>5</v>
-      </c>
-      <c r="E54">
-        <v>1</v>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">11X1</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">389.99</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FIRE BOLT-104</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FIRE BOLT</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VERTICAL</t>
-        </is>
-      </c>
-      <c r="D55">
-        <v>5</v>
-      </c>
-      <c r="E55">
-        <v>1</v>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5X10K</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">379.99</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DIYA-08 6X9</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DIYA</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">STUCKON</t>
-        </is>
-      </c>
-      <c r="D56">
-        <v>4</v>
-      </c>
-      <c r="E56">
-        <v>1</v>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6X9</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">639.99</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FIRE BOLT-155</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FIRE BOLT</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VERTICAL</t>
-        </is>
-      </c>
-      <c r="D57">
-        <v>3</v>
-      </c>
-      <c r="E57">
-        <v>1</v>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5X10K</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">359.99</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FIRE BOLT-02</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FIRE BOLT</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VERTICAL</t>
-        </is>
-      </c>
-      <c r="D58">
-        <v>1</v>
-      </c>
-      <c r="E58">
-        <v>1</v>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5X10K</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">449</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GSJ-22-L</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GSJ</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">STUCKON</t>
-        </is>
-      </c>
-      <c r="D59">
-        <v>1</v>
-      </c>
-      <c r="E59">
-        <v>1</v>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5X8</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">649</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SHOOT PHOTO - nothing in the archive</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TOTAL</t>
-        </is>
-      </c>
-      <c r="B60"/>
-      <c r="C60"/>
-      <c r="D60">
-        <v>3009</v>
-      </c>
-      <c r="E60"/>
-      <c r="F60"/>
-      <c r="G60"/>
-      <c r="H60"/>
-      <c r="I60"/>
+        <v>2031</v>
+      </c>
+      <c r="E53"/>
+      <c r="F53"/>
+      <c r="G53"/>
+      <c r="H53"/>
+      <c r="I53"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I60"/>
+  <autoFilter ref="A1:I53"/>
 </worksheet>
 </file>
 
@@ -35547,10 +35348,14 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="O51"/>
+          <t xml:space="preserve">SERIES ONLY</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 of 1</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -38696,7 +38501,11 @@
           <t xml:space="preserve">NO PHOTO</t>
         </is>
       </c>
-      <c r="O93"/>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 of 1</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -39294,7 +39103,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 of 5</t>
+          <t xml:space="preserve">0 of 2</t>
         </is>
       </c>
     </row>
@@ -39364,10 +39173,14 @@
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="O102"/>
+          <t xml:space="preserve">SERIES ONLY</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 of 3</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -39660,10 +39473,14 @@
       </c>
       <c r="N106" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="O106"/>
+          <t xml:space="preserve">SERIES ONLY</t>
+        </is>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 of 1</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -41531,10 +41348,14 @@
       </c>
       <c r="N131" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="O131"/>
+          <t xml:space="preserve">OWN PHOTO</t>
+        </is>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 of 1</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -41602,10 +41423,14 @@
       </c>
       <c r="N132" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="O132"/>
+          <t xml:space="preserve">OWN PHOTO</t>
+        </is>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 of 2</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -41673,10 +41498,14 @@
       </c>
       <c r="N133" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="O133"/>
+          <t xml:space="preserve">OWN PHOTO</t>
+        </is>
+      </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 of 1</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -41744,10 +41573,14 @@
       </c>
       <c r="N134" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="O134"/>
+          <t xml:space="preserve">OWN PHOTO</t>
+        </is>
+      </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 of 1</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -43690,10 +43523,14 @@
       </c>
       <c r="N160" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="O160"/>
+          <t xml:space="preserve">SERIES ONLY</t>
+        </is>
+      </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 of 1</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -44436,7 +44273,7 @@
       </c>
       <c r="N170" t="inlineStr">
         <is>
-          <t xml:space="preserve">OWN PHOTO</t>
+          <t xml:space="preserve">SERIES ONLY</t>
         </is>
       </c>
       <c r="O170" t="inlineStr">
@@ -48941,7 +48778,7 @@
       </c>
       <c r="O230" t="inlineStr">
         <is>
-          <t xml:space="preserve">0 of 3</t>
+          <t xml:space="preserve">0 of 4</t>
         </is>
       </c>
     </row>
@@ -51786,7 +51623,7 @@
       </c>
       <c r="N268" t="inlineStr">
         <is>
-          <t xml:space="preserve">OWN PHOTO</t>
+          <t xml:space="preserve">SERIES ONLY</t>
         </is>
       </c>
       <c r="O268" t="inlineStr">
@@ -52236,7 +52073,7 @@
       </c>
       <c r="N274" t="inlineStr">
         <is>
-          <t xml:space="preserve">OWN PHOTO</t>
+          <t xml:space="preserve">SERIES ONLY</t>
         </is>
       </c>
       <c r="O274" t="inlineStr">
@@ -55311,7 +55148,7 @@
       </c>
       <c r="N315" t="inlineStr">
         <is>
-          <t xml:space="preserve">OWN PHOTO</t>
+          <t xml:space="preserve">SERIES ONLY</t>
         </is>
       </c>
       <c r="O315" t="inlineStr">
@@ -59511,7 +59348,7 @@
       </c>
       <c r="N371" t="inlineStr">
         <is>
-          <t xml:space="preserve">OWN PHOTO</t>
+          <t xml:space="preserve">SERIES ONLY</t>
         </is>
       </c>
       <c r="O371" t="inlineStr">
@@ -61086,10 +60923,14 @@
       </c>
       <c r="N392" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="O392"/>
+          <t xml:space="preserve">OWN PHOTO</t>
+        </is>
+      </c>
+      <c r="O392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 of 2</t>
+        </is>
+      </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
@@ -61157,10 +60998,14 @@
       </c>
       <c r="N393" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="O393"/>
+          <t xml:space="preserve">OWN PHOTO</t>
+        </is>
+      </c>
+      <c r="O393" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 of 2</t>
+        </is>
+      </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
@@ -61228,10 +61073,14 @@
       </c>
       <c r="N394" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="O394"/>
+          <t xml:space="preserve">OWN PHOTO</t>
+        </is>
+      </c>
+      <c r="O394" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 of 1</t>
+        </is>
+      </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
@@ -61299,10 +61148,14 @@
       </c>
       <c r="N395" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="O395"/>
+          <t xml:space="preserve">OWN PHOTO</t>
+        </is>
+      </c>
+      <c r="O395" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 of 1</t>
+        </is>
+      </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
@@ -61373,7 +61226,11 @@
           <t xml:space="preserve">NO PHOTO</t>
         </is>
       </c>
-      <c r="O396"/>
+      <c r="O396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 of 1</t>
+        </is>
+      </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -61441,10 +61298,14 @@
       </c>
       <c r="N397" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="O397"/>
+          <t xml:space="preserve">OWN PHOTO</t>
+        </is>
+      </c>
+      <c r="O397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 of 2</t>
+        </is>
+      </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
@@ -61515,7 +61376,11 @@
           <t xml:space="preserve">NO PHOTO</t>
         </is>
       </c>
-      <c r="O398"/>
+      <c r="O398" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 of 1</t>
+        </is>
+      </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
@@ -61583,10 +61448,14 @@
       </c>
       <c r="N399" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="O399"/>
+          <t xml:space="preserve">OWN PHOTO</t>
+        </is>
+      </c>
+      <c r="O399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 of 1</t>
+        </is>
+      </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
@@ -61654,10 +61523,14 @@
       </c>
       <c r="N400" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="O400"/>
+          <t xml:space="preserve">OWN PHOTO</t>
+        </is>
+      </c>
+      <c r="O400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 of 2</t>
+        </is>
+      </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
@@ -61725,10 +61598,14 @@
       </c>
       <c r="N401" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO PHOTO</t>
-        </is>
-      </c>
-      <c r="O401"/>
+          <t xml:space="preserve">OWN PHOTO</t>
+        </is>
+      </c>
+      <c r="O401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 of 1</t>
+        </is>
+      </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
@@ -65840,7 +65717,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>394</v>
+        <v>398</v>
       </c>
     </row>
     <row r="7">
@@ -65850,7 +65727,7 @@
         </is>
       </c>
       <c r="B7">
-        <v>36</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8">

</xml_diff>